<commit_message>
Add opportunity Forecast Category field (Uncommitted/Best Case/Committed)
Forecast category is an opportunity-level field (the MSX forecast object) - the opportunity moves Uncommitted -> Best Case -> Committed as milestones complete. Distinct from milestone customer commitment (execution/readiness).

- packages/shared: FORECAST_CATEGORIES list + CHOICES entry
- prisma: forecastCategory String? on Opportunity
- api: Zod createOpportunitySchema (flows to update + agent Create/UpdateOpportunity approval actions); service persists via spread
- web: form select, detail view, list column + filter, approval card field, badge colors
- workbook: Forecast Category column on Opportunity sheet (values by sales stage) + mapping
- openapi: forecastCategory on OpportunityInput + inline action schema; regenerated JSON

Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/MSX_Mirror_Necessary_Tables_Import_10_More_Entries.xlsx
+++ b/data/MSX_Mirror_Necessary_Tables_Import_10_More_Entries.xlsx
@@ -7208,7 +7208,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:R16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7262,6 +7262,9 @@
       <c r="Q1" t="str">
         <v>Last Updated</v>
       </c>
+      <c r="R1" t="str">
+        <v>Forecast Category</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -7315,6 +7318,9 @@
       <c r="Q2" t="str">
         <v>2026-07-03</v>
       </c>
+      <c r="R2" t="str">
+        <v>Uncommitted</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -7368,6 +7374,9 @@
       <c r="Q3" t="str">
         <v>2026-07-03</v>
       </c>
+      <c r="R3" t="str">
+        <v>Uncommitted</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -7418,6 +7427,9 @@
       <c r="Q4" t="str">
         <v>2026-07-03</v>
       </c>
+      <c r="R4" t="str">
+        <v>Best Case</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -7471,6 +7483,9 @@
       <c r="Q5" t="str">
         <v>2026-07-03</v>
       </c>
+      <c r="R5" t="str">
+        <v>Committed</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -7524,6 +7539,9 @@
       <c r="Q6" t="str">
         <v>2026-07-03</v>
       </c>
+      <c r="R6" t="str">
+        <v>Committed</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -7577,6 +7595,9 @@
       <c r="Q7">
         <v>46210</v>
       </c>
+      <c r="R7" t="str">
+        <v>Uncommitted</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -7630,6 +7651,9 @@
       <c r="Q8">
         <v>46210</v>
       </c>
+      <c r="R8" t="str">
+        <v>Best Case</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -7683,6 +7707,9 @@
       <c r="Q9">
         <v>46210</v>
       </c>
+      <c r="R9" t="str">
+        <v>Uncommitted</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -7736,6 +7763,9 @@
       <c r="Q10">
         <v>46210</v>
       </c>
+      <c r="R10" t="str">
+        <v>Uncommitted</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -7789,6 +7819,9 @@
       <c r="Q11">
         <v>46210</v>
       </c>
+      <c r="R11" t="str">
+        <v>Committed</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -7842,6 +7875,9 @@
       <c r="Q12">
         <v>46210</v>
       </c>
+      <c r="R12" t="str">
+        <v>Committed</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -7892,6 +7928,9 @@
       <c r="Q13">
         <v>46210</v>
       </c>
+      <c r="R13" t="str">
+        <v>Uncommitted</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -7945,6 +7984,9 @@
       <c r="Q14">
         <v>46210</v>
       </c>
+      <c r="R14" t="str">
+        <v>Best Case</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -7998,6 +8040,9 @@
       <c r="Q15">
         <v>46210</v>
       </c>
+      <c r="R15" t="str">
+        <v>Committed</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -8048,11 +8093,14 @@
       <c r="Q16">
         <v>46210</v>
       </c>
+      <c r="R16" t="str">
+        <v>Uncommitted</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R16"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>